<commit_message>
Operator passwords from the Sheet, factory WiFi via secrets.h
- Login screen: password field with keyboard; checked against column B of
  the Operators tab (last synced copy, so it also works offline);
  empty password in the Sheet = no password
- Sheets sync reads Operators!A2:B11 and caches the passwords
- secrets.h can define WIFI_SSID / WIFI_PASS, used until other
  credentials are saved on the Admin screen
- Template and setup guide updated with the password column

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LXTvxhwrQucbbkRLzNXi3e
</commit_message>
<xml_diff>
--- a/docs/Contactor_IQC_Sheet_Template.xlsx
+++ b/docs/Contactor_IQC_Sheet_Template.xlsx
@@ -768,10 +768,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -780,9 +781,15 @@
           <t>Operator Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Max 10 names, one per row from A2. Shown in the login dropdown.</t>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Operator Password</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Max 10 operators. Password is checked on the login screen; leave it empty for no password.</t>
         </is>
       </c>
     </row>
@@ -792,6 +799,11 @@
           <t>Operator 1</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>password 1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -799,11 +811,21 @@
           <t>Operator 2</t>
         </is>
       </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>password 2</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Operator 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>password 3</t>
         </is>
       </c>
     </row>
@@ -980,9 +1002,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -993,7 +1013,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Operators  : names shown in the login dropdown (max 10).</t>
+          <t>Operators  : names (column A) and passwords (column B) for the login screen, max 10.</t>
         </is>
       </c>
     </row>
@@ -1004,9 +1024,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -1056,9 +1074,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix test-screen flicker, pause Sheet uploads during tests, 5-cycle Results
- Test grid uses one object per cell instead of lv_table, so a value change
  redraws only that cell (~40x less frame-buffer traffic while running)
- Sheet uploads and syncs wait while a test runs; NEXT BATCH uploads them
- MAX_CYCLES 5: Results template and header TSV now end at 5- Release (43 cols)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LXTvxhwrQucbbkRLzNXi3e
</commit_message>
<xml_diff>
--- a/docs/Contactor_IQC_Sheet_Template.xlsx
+++ b/docs/Contactor_IQC_Sheet_Template.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -766,6 +766,13 @@
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Stagger = delay between the start of consecutive channels (keeps in-rush currents from overlapping).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cycles: 1 to 5 (the Results tab has columns for 5 cycles).</t>
         </is>
       </c>
     </row>
@@ -852,7 +859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ1"/>
+  <dimension ref="A1:AQ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1151,181 +1158,6 @@
           <t>5- Release</t>
         </is>
       </c>
-      <c r="AR1" s="6" t="inlineStr">
-        <is>
-          <t>6- Open</t>
-        </is>
-      </c>
-      <c r="AS1" s="6" t="inlineStr">
-        <is>
-          <t>6- Inrush (A)</t>
-        </is>
-      </c>
-      <c r="AT1" s="6" t="inlineStr">
-        <is>
-          <t>6- Inrush P/F</t>
-        </is>
-      </c>
-      <c r="AU1" s="6" t="inlineStr">
-        <is>
-          <t>6- Cont (A)</t>
-        </is>
-      </c>
-      <c r="AV1" s="6" t="inlineStr">
-        <is>
-          <t>6- Cont P/F</t>
-        </is>
-      </c>
-      <c r="AW1" s="6" t="inlineStr">
-        <is>
-          <t>6- Continuity</t>
-        </is>
-      </c>
-      <c r="AX1" s="6" t="inlineStr">
-        <is>
-          <t>6- Release</t>
-        </is>
-      </c>
-      <c r="AY1" s="6" t="inlineStr">
-        <is>
-          <t>7- Open</t>
-        </is>
-      </c>
-      <c r="AZ1" s="6" t="inlineStr">
-        <is>
-          <t>7- Inrush (A)</t>
-        </is>
-      </c>
-      <c r="BA1" s="6" t="inlineStr">
-        <is>
-          <t>7- Inrush P/F</t>
-        </is>
-      </c>
-      <c r="BB1" s="6" t="inlineStr">
-        <is>
-          <t>7- Cont (A)</t>
-        </is>
-      </c>
-      <c r="BC1" s="6" t="inlineStr">
-        <is>
-          <t>7- Cont P/F</t>
-        </is>
-      </c>
-      <c r="BD1" s="6" t="inlineStr">
-        <is>
-          <t>7- Continuity</t>
-        </is>
-      </c>
-      <c r="BE1" s="6" t="inlineStr">
-        <is>
-          <t>7- Release</t>
-        </is>
-      </c>
-      <c r="BF1" s="6" t="inlineStr">
-        <is>
-          <t>8- Open</t>
-        </is>
-      </c>
-      <c r="BG1" s="6" t="inlineStr">
-        <is>
-          <t>8- Inrush (A)</t>
-        </is>
-      </c>
-      <c r="BH1" s="6" t="inlineStr">
-        <is>
-          <t>8- Inrush P/F</t>
-        </is>
-      </c>
-      <c r="BI1" s="6" t="inlineStr">
-        <is>
-          <t>8- Cont (A)</t>
-        </is>
-      </c>
-      <c r="BJ1" s="6" t="inlineStr">
-        <is>
-          <t>8- Cont P/F</t>
-        </is>
-      </c>
-      <c r="BK1" s="6" t="inlineStr">
-        <is>
-          <t>8- Continuity</t>
-        </is>
-      </c>
-      <c r="BL1" s="6" t="inlineStr">
-        <is>
-          <t>8- Release</t>
-        </is>
-      </c>
-      <c r="BM1" s="6" t="inlineStr">
-        <is>
-          <t>9- Open</t>
-        </is>
-      </c>
-      <c r="BN1" s="6" t="inlineStr">
-        <is>
-          <t>9- Inrush (A)</t>
-        </is>
-      </c>
-      <c r="BO1" s="6" t="inlineStr">
-        <is>
-          <t>9- Inrush P/F</t>
-        </is>
-      </c>
-      <c r="BP1" s="6" t="inlineStr">
-        <is>
-          <t>9- Cont (A)</t>
-        </is>
-      </c>
-      <c r="BQ1" s="6" t="inlineStr">
-        <is>
-          <t>9- Cont P/F</t>
-        </is>
-      </c>
-      <c r="BR1" s="6" t="inlineStr">
-        <is>
-          <t>9- Continuity</t>
-        </is>
-      </c>
-      <c r="BS1" s="6" t="inlineStr">
-        <is>
-          <t>9- Release</t>
-        </is>
-      </c>
-      <c r="BT1" s="6" t="inlineStr">
-        <is>
-          <t>10- Open</t>
-        </is>
-      </c>
-      <c r="BU1" s="6" t="inlineStr">
-        <is>
-          <t>10- Inrush (A)</t>
-        </is>
-      </c>
-      <c r="BV1" s="6" t="inlineStr">
-        <is>
-          <t>10- Inrush P/F</t>
-        </is>
-      </c>
-      <c r="BW1" s="6" t="inlineStr">
-        <is>
-          <t>10- Cont (A)</t>
-        </is>
-      </c>
-      <c r="BX1" s="6" t="inlineStr">
-        <is>
-          <t>10- Cont P/F</t>
-        </is>
-      </c>
-      <c r="BY1" s="6" t="inlineStr">
-        <is>
-          <t>10- Continuity</t>
-        </is>
-      </c>
-      <c r="BZ1" s="6" t="inlineStr">
-        <is>
-          <t>10- Release</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:BZ100000">

</xml_diff>

<commit_message>
Continuity check for 4-pin contactors, chosen per model from the Specs sheet (0.5.0)
- Specs tab: new column M "Continuity" (Yes / No). Yes = feedback contact
  is checked and the HMI shows CLOSE / OPEN; No (2-pin) shows -NA-.
- Rig board firmware: reads feedback contacts on GPIO 1, 2, 10, 11, 12
  (contact to GND, internal pull-up), 5 ms debounce, latches any opening
  since the last stats reset; status packet version 2 carries both flags.
- HMI: accepts packet version 1 or 2, uses the contacts only for models with
  Continuity = Yes, refuses START if such a model is selected and the rig
  firmware has no contact inputs. Setup > Specs shows the Continuity column.
- Template xlsx and setup docs updated; rig README has the wiring.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LXTvxhwrQucbbkRLzNXi3e
</commit_message>
<xml_diff>
--- a/docs/Contactor_IQC_Sheet_Template.xlsx
+++ b/docs/Contactor_IQC_Sheet_Template.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -495,6 +495,7 @@
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -558,6 +559,11 @@
           <t>Stagger (ms)</t>
         </is>
       </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Continuity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -598,6 +604,11 @@
       <c r="L2" s="2" t="n">
         <v>1500</v>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -642,6 +653,11 @@
       <c r="L3" s="2" t="n">
         <v>1500</v>
       </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -682,6 +698,11 @@
       <c r="L4" s="2" t="n">
         <v>1500</v>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -726,7 +747,14 @@
       <c r="L5" s="2" t="n">
         <v>1500</v>
       </c>
-    </row>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -776,7 +804,19 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Continuity = Yes for 4-pin contactors (feedback contact wired to the rig): HMI shows CLOSE / OPEN. No = 2-pin, shows -NA-.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="M2:M9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Continuity on every contactor: main terminals OPEN before ON, CLOSE while ON
- Removes the per-model Specs "Continuity" column: every contactor is tested.
- Contin. OFF (was Open): main terminals must be OPEN and coil current ~0
  before the relay switches on. Contin. ON (was Continuity): terminals must
  stay CLOSE for the whole averaging window. Release check kept.
- Test screen and Results show the terminal state (OPEN / CLOSE), green when
  expected, red when not. Fail steps: "Contin OFF: CLOSE", "Contin OFF:
  current", "Contin ON: OPEN", "Release: CLOSE", "Release: current".
- START is refused if the rig board firmware cannot read continuity.
- Results header, template xlsx and docs renamed; rig README has the
  main-terminal wiring (GPIO 1, 2, 10, 11, 12, 2.2k pull-up to 3V3).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LXTvxhwrQucbbkRLzNXi3e
</commit_message>
<xml_diff>
--- a/docs/Contactor_IQC_Sheet_Template.xlsx
+++ b/docs/Contactor_IQC_Sheet_Template.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -559,11 +559,6 @@
           <t>Stagger (ms)</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
-        <is>
-          <t>Continuity</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -604,11 +599,6 @@
       <c r="L2" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -653,11 +643,6 @@
       <c r="L3" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -698,11 +683,6 @@
       <c r="L4" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -747,14 +727,7 @@
       <c r="L5" s="2" t="n">
         <v>1500</v>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="6"/>
-    <row r="7"/>
+    </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -804,19 +777,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Continuity = Yes for 4-pin contactors (feedback contact wired to the rig): HMI shows CLOSE / OPEN. No = 2-pin, shows -NA-.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="M2:M9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1025,7 +986,7 @@
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>1- Open</t>
+          <t>1- Contin. OFF</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
@@ -1050,7 +1011,7 @@
       </c>
       <c r="N1" s="6" t="inlineStr">
         <is>
-          <t>1- Continuity</t>
+          <t>1- Contin. ON</t>
         </is>
       </c>
       <c r="O1" s="6" t="inlineStr">
@@ -1060,7 +1021,7 @@
       </c>
       <c r="P1" s="6" t="inlineStr">
         <is>
-          <t>2- Open</t>
+          <t>2- Contin. OFF</t>
         </is>
       </c>
       <c r="Q1" s="6" t="inlineStr">
@@ -1085,7 +1046,7 @@
       </c>
       <c r="U1" s="6" t="inlineStr">
         <is>
-          <t>2- Continuity</t>
+          <t>2- Contin. ON</t>
         </is>
       </c>
       <c r="V1" s="6" t="inlineStr">
@@ -1095,7 +1056,7 @@
       </c>
       <c r="W1" s="6" t="inlineStr">
         <is>
-          <t>3- Open</t>
+          <t>3- Contin. OFF</t>
         </is>
       </c>
       <c r="X1" s="6" t="inlineStr">
@@ -1120,7 +1081,7 @@
       </c>
       <c r="AB1" s="6" t="inlineStr">
         <is>
-          <t>3- Continuity</t>
+          <t>3- Contin. ON</t>
         </is>
       </c>
       <c r="AC1" s="6" t="inlineStr">
@@ -1130,7 +1091,7 @@
       </c>
       <c r="AD1" s="6" t="inlineStr">
         <is>
-          <t>4- Open</t>
+          <t>4- Contin. OFF</t>
         </is>
       </c>
       <c r="AE1" s="6" t="inlineStr">
@@ -1155,7 +1116,7 @@
       </c>
       <c r="AI1" s="6" t="inlineStr">
         <is>
-          <t>4- Continuity</t>
+          <t>4- Contin. ON</t>
         </is>
       </c>
       <c r="AJ1" s="6" t="inlineStr">
@@ -1165,7 +1126,7 @@
       </c>
       <c r="AK1" s="6" t="inlineStr">
         <is>
-          <t>5- Open</t>
+          <t>5- Contin. OFF</t>
         </is>
       </c>
       <c r="AL1" s="6" t="inlineStr">
@@ -1190,7 +1151,7 @@
       </c>
       <c r="AP1" s="6" t="inlineStr">
         <is>
-          <t>5- Continuity</t>
+          <t>5- Contin. ON</t>
         </is>
       </c>
       <c r="AQ1" s="6" t="inlineStr">
@@ -1301,14 +1262,14 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Fail Step    step that failed, e.g. In-rush, Continuous current, Continuity, Release, Open</t>
+          <t xml:space="preserve">  Fail Step    step that failed, e.g. In-rush, Continuous current, Contin ON: OPEN, Contin OFF: CLOSE, Release: CLOSE</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  n- ...       results of cycle n (Open, Inrush A, Inrush P/F, Cont A, Cont P/F, Continuity, Release)</t>
+          <t xml:space="preserve">  n- ...       results of cycle n (Contin. OFF, Inrush A, Inrush P/F, Cont A, Cont P/F, Contin. ON, Release)</t>
         </is>
       </c>
     </row>

</xml_diff>